<commit_message>
Expand Kaptai resort list to 19 stays + houseboats/operators
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164MYEZuLZ1BUVpVHt4sH1c
</commit_message>
<xml_diff>
--- a/Kaptai_Rangamati_Resorts.xlsx
+++ b/Kaptai_Rangamati_Resorts.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Resorts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Houseboats &amp; Operators" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes &amp; Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,19 +467,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,47 +494,67 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Resort Name</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Area / Location</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Phone / Booking</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Facebook / Website</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Facebook / Social</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Approx. Price</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Google Maps Link</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes (for 30 people)</t>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes for 30 people</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Verification status</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Google Maps (search link)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Sources</t>
         </is>
       </c>
     </row>
@@ -544,42 +569,62 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Kaptai side (Kaptaimukh)</t>
+          <t>Lakeside resort</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Jeebtali-Log Gate Link Road, Kaptaimukh, Kaptai, Rangamati/Chattogram</t>
+          <t>Kaptaimukh / Jeebtoli, Kaptai</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>01859-778065 (advance booking)</t>
+          <t>Jeebtali-Log Gate Link Road, Kaptaimukh, Kaptai, Chattogram 4530</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Email listed on tourtobangladesh.com (address hidden in source)</t>
+          <t>01859-778065 (booking); 01550-322448 (2nd source, conflict)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Obfuscated in sources - not seen</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>hotelresortbd.com/lakeshore-resort/</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/LakeshoreResortKaptai</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Tk 4,500-6,500/night; ~15 lakeside cottages</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Lakeshore%20Resort%20Kaptai%20Rangamati</t>
-        </is>
-      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Reported by 4 sources; good fit for a 30-person group (multiple cottages) - confirm total capacity</t>
+          <t>Room ~Tk 4,500-9,000; ~Tk 5,000 w/ breakfast; whole resort ~Tk 40,000/night (one source); kayak Tk 200/hr</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>~15 cottages, AC rooms, glass-house lobby, pool, 200ft hanging bridge; whole-resort booking reportedly offered - BEST FIT for 30</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Multiple sources; phones conflict</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Lakeshore%20Resort%20Kaptai</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>tripadvisor d7928494; tourtobangladesh.com; marketbangladesh.com; asiafirms</t>
         </is>
       </c>
     </row>
@@ -594,42 +639,62 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Island in Kaptai Lake, ~10 min boat from Kaptai main ghat</t>
+          <t>Island resort</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Lake, Kaptai, Rangamati (boat access)</t>
+          <t>Island ~10 min boat from Kaptai main ghat</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>01769-322183; 01797-322172 / 01797-322173 (source printed 0179322172/3); 01746-191421</t>
+          <t>Kaptai Lake, Kaptai, Rangamati</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not found - verify</t>
+          <t>01769-322183; 01769-322182; 01746-191421 / 01847-191421; 0179322172/3 (probably missing digit) - all unverified</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/p/Lakeview-Island-Resort-100086979506274</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Not found - verify</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Resort, houseboat, boat club, playground; 25% advance reportedly required</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Phones conflict - call FB page number</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20View%20Island%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Resort, houseboat, boat club, playground. Numbers vary across sources - call to confirm</t>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>lrbtravelteam.com; vromonguide; FB</t>
         </is>
       </c>
     </row>
@@ -639,47 +704,67 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Bargee Lake Valley (Bargee/Bargi)</t>
+          <t>Divine Lake Island Resort</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Boradam / Manikchori Mukh, Asambosti-Kaptai Road, Rangamati Sadar</t>
+          <t>Island resort (6 acre)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Dellye Bagan, Manikchori Mukh, Boradam, Asambosti-Kaptai Road, Rangamati Sadar, Rangamati 4500</t>
+          <t>Near Asambosti bridge, Kaptai Road, Rangamati</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Not found - see Facebook page</t>
+          <t>Kaptai Road, Ashambosti, Rangamati 4500 (boat-only; call reception from Asambosti pier)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>01958-054408; 01611-585887 (conflict)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/p/Bargee-Lake-Valley-100068030345250 ; amarlodge.com/hotels/292/bd/Bargee-Lake-Valley</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Budget resort (price not found)</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
+          <t>divinelakeisland.com</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/divinelakeisland</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Eco-resort on lake shore with water rides; also has a Camping page</t>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Cottages + floating rooms; read website /terms for group policy</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Phones conflict</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Kaptai%20Road%20Ashambosti%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>divinelakeisland.com; avijatrik.org; asiafirms</t>
         </is>
       </c>
     </row>
@@ -689,47 +774,67 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Divine Lake Island Resort</t>
+          <t>Hill Taj Resort / The Grand Hill Taj</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Island near Asambosti pier, Rangamati</t>
+          <t>Island resort + water park</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Road, Ashambosti, Rangamati 4500 (boat-only; call reception from Asambosti pier, boat within ~30 min)</t>
+          <t>Rangamati Sadar (island)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>01958-054408; 01611-585887</t>
+          <t>C.O. Office Ghat, Furfura Tila, Rangamati 4500</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1870-701892 (labelled 'merchant account' - may be payment number)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>divinelakeisland.com ; facebook.com/divinelakeisland</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Not found - verify</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Kaptai%20Road%20Ashambosti%20Rangamati</t>
+          <t>parjatanbd.com hotel id 402</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/thegrandhilltaj</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Secluded island resort; check group capacity and terms at website</t>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Pool + adjacent Happy Island water park</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Booking number doubtful</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hill%20Taj%20Resort%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>tripadvisor d16858882; bdbooking; bd-info</t>
         </is>
       </c>
     </row>
@@ -739,47 +844,67 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Hill Taj Resort / The Grand Hill Taj</t>
+          <t>Wildwood Island Resort</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Island in Kaptai Lake, Rangamati Sadar</t>
+          <t>Island resort (luxury)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>C.O. Office Ghat / Furfura Tila area; Kaptai Lake, Rangamati Sadar, Rangamati 4500</t>
+          <t>Diglibagh, Rangamati Sadar</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>+880 1870-701892 (booking)</t>
+          <t>Diglibagh, Rangamati 4500</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1833-334309</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/thegrandhilltaj ; parjatanbd.com hotel id 402</t>
+          <t>wildwoodislandresort@gmail.com</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not found - verify</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hill%20Taj%20Resort%20Rangamati</t>
+          <t>wildwoodisland.com</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/Wildwoodislandresort</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Island resort with pool and adjacent Happy Island water park</t>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Lake-view rooms; also on Agoda/Expedia</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Seen in 3 agents' results</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Wildwood%20Island%20Resort%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>wildwoodisland.com; insidebangla; tripadvisor</t>
         </is>
       </c>
     </row>
@@ -789,47 +914,67 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Aronnak (Aronnok) Holiday Resort</t>
+          <t>Nilanjana Boat Club &amp; Resort</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Near Circuit House / Infantry Brigade, Rangamati Sadar</t>
+          <t>Floating + hilltop cottages</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Near Infantry Brigade, Rangamati Sadar, Rangamati, Chattogram</t>
+          <t>Asambosti, Kaptai Lake (10 min from Tabalchari ghat)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>+880 1769-312021; 01669-312022</t>
+          <t>Asham Bosti, Kaptai Lake, Rangamati</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>arannokhtj45@gmail.com</t>
+          <t>01911-060900; 01833-334311 (conflict)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/AronnakHolidayCottage ; facebook.com/aronnok.mk</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Tk 5,000-10,000/night</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
+          <t>nilanjanaboatclubresort.reservehotel.net</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/nilanjanaboatclubandresort</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Lakeside cottages; Parjatan hotel id 404</t>
+          <t>Family suite Tk 16,000; 1N2D lake package Tk 10,000 (pick-up, kayak, breakfast)</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Capacity not found</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Phones conflict</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Nilanjana%20Boat%20Club%20and%20Resort%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>avijatrik.org; tripbangla; offerong</t>
         </is>
       </c>
     </row>
@@ -839,47 +984,67 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Parjatan Holiday Complex, Rangamati</t>
+          <t>Bargee Lake Valley (+ Camping)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Hanging Bridge Road, Rangamati town</t>
+          <t>Budget eco-resort</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hanging Bridge Rd, Rangamati Sadar</t>
+          <t>Boradam / Manikchori Mukh, Asambosti-Kaptai Rd</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>02-333371853 / +880-233-3371851; 01863-231185; 01991-139037</t>
+          <t>Dellye Bagan, Manikchori Mukh, Boradam, Rangamati Sadar 4500</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>See hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
+          <t>No own number found (only Take A Boat platform +880 9601-621641)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
+          <t>info@takeaboat.com (platform, not resort)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Tk 1,600-6,000/night</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Bargee-Lake-Valley-100068030345250 ; facebook.com/p/Bargee-Lake-Valley-Camping-Rangamati-100075681652008</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Government (BPC) hotel; easiest for official group booking</t>
+          <t>Budget; not found</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Water rides; capacity not found</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Contact via Facebook</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>amarlodge.com; takeaboat.com; adarbepari; trippainter</t>
         </is>
       </c>
     </row>
@@ -889,47 +1054,67 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Hotel Jum Palace</t>
+          <t>Aronnak (Aronnok) Holiday Resort</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>T&amp;T Area, Rangamati town</t>
+          <t>Lakeside cottages (Army-run)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>T&amp;T Area, Rangamati</t>
+          <t>Near Circuit House / Infantry Brigade, Rangamati Sadar</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>0351-61878; 01625-100000</t>
+          <t>Near Infantry Brigade, Rangamati Sadar</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>01769-312021; 01669-312022</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>arannokhtj45@gmail.com</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Tk 1,500-3,200/night</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
+          <t>parjatanbd.com hotel id 404</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/AronnakHolidayCottage ; facebook.com/aronnok.mk</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Hotel not resort; budget option</t>
+          <t>Tk 5,000-10,000/night</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>~4 VIP + 7 ordinary rooms (small for 30 - may need 2 places)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Consistent across sources</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>tripadvisor d7928494; bdbooking; mawbiz</t>
         </is>
       </c>
     </row>
@@ -939,47 +1124,67 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Hotel Shanghai International</t>
+          <t>Nisarga Pod House / Nisarga River Valley</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Central Rangamati</t>
+          <t>Pod cottages, glamping</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Rangamati town (near Hanging Bridge)</t>
+          <t>Shilchori, Kaptai (Karnaphuli bank)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Not found - see TripAdvisor listing</t>
+          <t>Shilchori, Kaptai upazila</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1829-806801; +880 1818-441100; +880 1628-378633</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor.com listing d10348460</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
+          <t>nisargapodhouse.com</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Nisarga-Pod-House-Kaptai-100063674163695 ; facebook.com/p/Nisarga-River-Valley-Pod-House-Kaptai-100083223187517</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>28 rooms, free breakfast (per TripAdvisor)</t>
+          <t>Tk 5,000/2 people incl. meals + kayak; Tk 6,000/3 people</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Capacity not found; barbecue, kayaking; Dhaka Tribune feature</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Multiple numbers - confirm</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Nisarga%20Pod%20House%20Kaptai</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>dhakatribune.com; trip.com; nisargapodhouse.com</t>
         </is>
       </c>
     </row>
@@ -994,42 +1199,62 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Lake, Rangamati</t>
+          <t>Camping, bamboo cottages</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Not found - see website</t>
+          <t>Near Kaptai Lake, Rangamati</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Not found - see website</t>
+          <t>Not found (see website)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not found (FB post mentions WhatsApp)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
           <t>kaptaiecovalley.com</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>From Tk 1,200/night (camping/bamboo cottages)</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/KaptaiEcoValley</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>From Tk 1,200/night</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Tents/cottages, bonfire, kayaking - good for large groups</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Phone missing</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Eco%20Valley</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Camping, bamboo cottages, kayaking</t>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>kaptaiecovalley.com; tourfo.com</t>
         </is>
       </c>
     </row>
@@ -1039,27 +1264,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Polwel Park &amp; Cottage</t>
+          <t>Kaptai Riverview Camping Point (KRCP)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Beside Kaptai Lake</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Kaptaimukh, opposite Kaptai Union Parishad Office</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Kaptaimukh, Kaptai</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1795-166199; +880 1816-110300</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1072,14 +1297,34 @@
           <t>Not found</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20%26%20Cottage%20Kaptai</t>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/KCP1BD</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Mentioned in search results only - verify existence/contact</t>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Camping - possible for big group</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>FB snippet only</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Riverview%20Camping%20Point%20Kaptaimukh</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/KCP1BD</t>
         </is>
       </c>
     </row>
@@ -1089,64 +1334,652 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Rangadip Resort Rangamati</t>
+          <t>Lake Paradise Picnic Spot &amp; Resort</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>Picnic spot + cottages (Navy-linked page)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Kaptai</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>lakeparadisebd.com</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/NavyPicnicSpotKaptai</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Lake/hill-view cottage rooms</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>No contact found</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20Paradise%20Kaptai</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>lakeparadisebd.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Green River View Hotel / Guest House</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Guest house</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Kaptaimukh, Kaptai</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Kaptaimukh, Chattogram</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>01889-777830; 01819-351050</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/greenriverviewkaptaihotel</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Lake/hill view</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>From Bangla snippet</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Green%20River%20View%20Kaptai%20Hotel</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>vromontrips/vromonguide snippet; FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Polwel Park &amp; Cottage</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Resort (run by Rangamati District Police)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>DC Bungalow Road, Rangamati</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>DC Bungalow Road, Rangamati</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>01877-725541; 01877-725542</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>polwelresort@gmail.com</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>polwelpark.com</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Luxury, secured</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Snippet only</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20and%20Cottage%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>tripsilo; vromonguide snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Parjatan Holiday Complex Rangamati</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Govt (BPC) hotel</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Hanging Bridge Road, Rangamati town</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Hanging Bridge Rd, Rangamati Sadar</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>02-333371853 / 02-333371851; 01863-231185; 01991-139037; 0351-63126</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Tk 1,600-6,000/night</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Easiest official group booking</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Consistent</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>hotels.gov.bd; tripadvisor</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Jum Palace</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Opp. post office, T&amp;T Area, Rangamati</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>T&amp;T Area, Rangamati</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>0351-61878; 01625-100000</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>See website</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>jumpalace.com</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/HotelJumPalacebd</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Tk 1,500-3,200/night</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Consistent</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>jumpalace.com; snippets</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Shanghai International</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Central Rangamati</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati town</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>28 rooms, free breakfast</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>No contact found</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>tripadvisor d10348460</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Rangadip / Ranga Dwip Resort</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Resort</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Unverified name</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rangadip%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Listed on TripAdvisor as nearest hotel to Kaptai Lake - verify</t>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>tripadvisor listing mention</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Raina Togun Eco Resort</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Eco resort</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Kaptai</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Bangla snippet only</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>UNVERIFIED - follow-up search found nothing</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Raina%20Togun%20Eco%20Resort%20Kaptai</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>goofly24/vromonguide snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Rajmahal International</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Seen, not researched</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Rajmahal%20International%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>search snippet</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1158,65 +1991,467 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Website / Source</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Capacity / Price</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Royal Adventure (double-decker houseboat)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Houseboat</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Kaptai Lake, Rangamati</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>+880 1711-336825; 01402-288573; 01678-076361; 01911-060900 (also Nilanjana's - verify)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>bdcruise.com/royal-adventure/ ; hoihullorholidays.com/royal-adventure/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/RoyalAdventurer</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>8 rooms x 4 = up to 32 people; 2D1N package; price Tk 85,000 (6 ppl) - 115,000 (12 ppl) per source</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Best houseboat fit for 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Promodini Boat Life (Avijatrik Tourism)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Houseboat x2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Kaptai Lake, Rangamati</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>avijatrik.org/tour/promodini-boat-life</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Promodini-1 sleeps 6 + Promodini-2 sleeps 10 = 16 only</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Too small alone for 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BD Cruise</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Tour operator/houseboats</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati-Kaptai</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>bdcruise.com/rangamati-kaptai-lake/</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Ask for 30-person quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GoZayaan</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Tour operator</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>gozayaan.com/destination/rangamati-tour-package</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Package quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Galaxy Holidays BD</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Tour operator</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>galaxyholidaysbd.com/package/Rangamati-Chittagong</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Package quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ITS Holidays Ltd</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tour operator</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>itsholidaysltd.com/rangamati-and-kaptai-tour-package</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Package quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Bangladesh Travel and Tours / Hoihullor Holidays</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Tour operators</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>bangladeshtravelandtours.com ; hoihullorholidays.com</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Houseboat packages</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>General Rangamati hotel &amp; boat booking line</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Unverified number</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>+880 1841-862600 (single Bangla snippet)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Data caveats (please read)</t>
+          <t>Research log (autoresearch-style loop: metric = distinct resorts found; keep new/verified, discard duplicates)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Compiled from web search snippets (TripAdvisor, Facebook pages, Bangladesh Parjatan, travel blogs) on 30 Sep 2026.</t>
+          <t>Round 1 (single search): 12 entries. Round 2 (4 parallel agents: Facebook/social, YouTube/blogs, verification, Kaptai-upazila): 19 stay entries + 8 houseboat/operator entries after de-duplication.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Several travel-guide sites (vromonguide, bd-info, etc.) were blocked, so pages could not be opened; 'Not found' means not seen, not that none exists.</t>
+          <t>LIMITS: Facebook, YouTube, Instagram, X, TripAdvisor and most Bangla travel blogs were blocked from this environment (proxy); only search-result snippets were readable. YouTube/X gave nothing usable.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Phone numbers differ between sources; CALL AND CONFIRM before paying any advance. Prices are old blog figures.</t>
+          <t>No coordinates or exact Google Maps place URLs found; the Maps links are name searches - confirm the pin.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Google Maps links are search links by resort name (not exact pin coordinates); open and confirm the right pin.</t>
+          <t>Phones conflict for Lakeshore, Lake View Island, Divine Lake Island, Nilanjana; Hill Taj number may be a payment number; Bargee has only a platform number. CALL AND CONFIRM before advance payment.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>For 30 people: ask each resort about total room/cottage capacity, group discount, meals, boat transfer, and lake-boat hire.</t>
+          <t>Prices are old blog/listing figures. Ask for 30-person group rate, meals, boat transfer, whole-resort booking.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Island resorts (Lake View, Divine, Hill Taj) need boat transfer - budget extra time/cost.</t>
+          <t>Not opened (blocked; try on your own network): vromonguide.com/hotels-and-resorts-in-rangamati, bd-info.com/rangamati-hotel-resort-list, ratekom.com list, goofly24 blog, resortian.com/blog/kaptai-lake-resorts, TripAdvisor hotels near Kaptai Lake.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Sources: tripadvisor.com, facebook.com pages listed, hotels.gov.bd, parjatanbd.com, divinelakeisland.com, kaptaiecovalley.com, tourtobangladesh.com</t>
+          <t>Shortlist for 30 people: Lakeshore (whole-resort), Royal Adventure houseboat (32 cap.), Kaptai Eco Valley (camping), Parjatan Holiday Complex (official), or split between Aronnak + another.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Round 3: fill gaps, add more resorts, hotels and houseboat operators
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164MYEZuLZ1BUVpVHt4sH1c
</commit_message>
<xml_diff>
--- a/Kaptai_Rangamati_Resorts.xlsx
+++ b/Kaptai_Rangamati_Resorts.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resorts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Houseboats &amp; Operators" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resorts &amp; Hotels" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Houseboats &amp; Transport" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Notes &amp; Log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -467,23 +467,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,7 +504,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Area / Location</t>
+          <t>Area</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -534,17 +534,17 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Approx. Price</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Notes for 30 people</t>
+          <t>Capacity / Notes for 30</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Verification status</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -584,17 +584,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>01859-778065 (booking); 01550-322448 (2nd source, conflict)</t>
+          <t>01859-778065 (most cited); 01550-322448 (asiafirms) - CONFLICT</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Obfuscated in sources - not seen</t>
+          <t>Obfuscated in sources</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>hotelresortbd.com/lakeshore-resort/</t>
+          <t>aronnok.com may be sister property (Aronnok &amp; Lakeshore)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -604,17 +604,17 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Room ~Tk 4,500-9,000; ~Tk 5,000 w/ breakfast; whole resort ~Tk 40,000/night (one source); kayak Tk 200/hr</t>
+          <t>Room ~Tk 5,000 (range 4,500-9,000); WHOLE RESORT ~Tk 40,000/night; kayak Tk 200/hr; entry Tk 50</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>~15 cottages, AC rooms, glass-house lobby, pool, 200ft hanging bridge; whole-resort booking reportedly offered - BEST FIT for 30</t>
+          <t>15 cottages, AC rooms, pool, restaurant/BBQ, 200ft hanging bridge; whole-resort booking - BEST FIT for 30</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Multiple sources; phones conflict</t>
+          <t>Multi-source; phones conflict</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor d7928494; tourtobangladesh.com; marketbangladesh.com; asiafirms</t>
+          <t>hotelresortbd.com; asiafirms; marketbangladesh; tourtobangladesh; tripbangla</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Lake View Island Resort</t>
+          <t>Lake View Island Resort (Army-run)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -644,17 +644,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Island ~10 min boat from Kaptai main ghat</t>
+          <t>Island ~10 min boat from Kaptai ghat</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Lake, Kaptai, Rangamati</t>
+          <t>Kaptai Lake, Kaptai (boat access)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>01769-322183; 01769-322182; 01746-191421 / 01847-191421; 0179322172/3 (probably missing digit) - all unverified</t>
+          <t>01769-322183; 01769-322182; 01746-191421 / 01847-191421; 0179322172/3 (malformed) - CONFLICT</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -669,22 +669,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/p/Lakeview-Island-Resort-100086979506274</t>
+          <t>facebook.com/kaptai.island2016 ; facebook.com/p/Lakeview-Island-Resort-100086979506274</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Civilian Tk 4,300/room/night; military Tk 1,025; 25% advance</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Resort, houseboat, boat club, playground; 25% advance reportedly required</t>
+          <t>Cottages, restaurant, houseboat, boat club; cottage count not found</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Phones conflict - call FB page number</t>
+          <t>Phones conflict</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>lrbtravelteam.com; vromonguide; FB</t>
+          <t>lrbtravelteam; tripadvisor d13974943; vromonguide</t>
         </is>
       </c>
     </row>
@@ -714,17 +714,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Near Asambosti bridge, Kaptai Road, Rangamati</t>
+          <t>Near Asambosti bridge, Kaptai Road</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Road, Ashambosti, Rangamati 4500 (boat-only; call reception from Asambosti pier)</t>
+          <t>Kaptai Road, Ashambosti, Rangamati 4500 (call reception at Asambosti pier; free shuttle boat ~30 min)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>01958-054408; 01611-585887 (conflict)</t>
+          <t>01611-585887 (2 sources); 01958-054408 (1 source)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>AC cottage Tk 6,000; bamboo cottage Tk 4,000-4,500</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Cottages + floating rooms; read website /terms for group policy</t>
+          <t>2 AC + 4 bamboo cottages (packages 2-15 people) - too small alone for 30</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -759,12 +759,12 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Kaptai%20Road%20Ashambosti%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Ashambosti%20Rangamati</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>divinelakeisland.com; avijatrik.org; asiafirms</t>
+          <t>avijatrik; tripsilo; booking.com</t>
         </is>
       </c>
     </row>
@@ -784,17 +784,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Rangamati Sadar (island)</t>
+          <t>Kaptai Lake, Rangamati Sadar</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>C.O. Office Ghat, Furfura Tila, Rangamati 4500</t>
+          <t>Kaptai Lake, Rangamati Sadar 4500; C.O. Office Ghat / Furfura Tila</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>+880 1870-701892 (labelled 'merchant account' - may be payment number)</t>
+          <t>+880 1600-343694; +880 1777-714621 (booking, per bd-info); +880 1870-701892 (merchant/payment?)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>parjatanbd.com hotel id 402</t>
+          <t>thegrandhilltaj.com</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -814,27 +814,27 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>OTA from ~US$74; 50% advance; free breakfast; free boat from city</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Pool + adjacent Happy Island water park</t>
+          <t>Treehouse, pool, 24/7 room dining; room count not found</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Booking number doubtful</t>
+          <t>Numbers conflict</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hill%20Taj%20Resort%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=The%20Grand%20Hill%20Taj%20Rangamati</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor d16858882; bdbooking; bd-info</t>
+          <t>bd-info; bdbooking; lrbtravelteam; thegrandhilltaj.com</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Island resort (luxury)</t>
+          <t>Luxury island resort</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -884,17 +884,17 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>~Tk 10,800-12,000/night (reviews); ~US$101 OTA</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Lake-view rooms; also on Agoda/Expedia</t>
+          <t>Villas: Luxury (Hill View), Superior, Junior, Family; count not found</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Seen in 3 agents' results</t>
+          <t>One source per contact</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>wildwoodisland.com; insidebangla; tripadvisor</t>
+          <t>insidebangla; tripadvisor d33959189; agoda</t>
         </is>
       </c>
     </row>
@@ -914,67 +914,67 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Nilanjana Boat Club &amp; Resort</t>
+          <t>Rangadip Resort</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Floating + hilltop cottages</t>
+          <t>Private island resort</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Asambosti, Kaptai Lake (10 min from Tabalchari ghat)</t>
+          <t>Rangamati</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Asham Bosti, Kaptai Lake, Rangamati</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>01911-060900; 01833-334311 (conflict)</t>
+          <t>+880 1327-475252; 01977-792001 (fragment)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>rangadipresort@gmail.com</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>nilanjanaboatclubresort.reservehotel.net</t>
+          <t>rangadipresort.com / rangadip.com</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/nilanjanaboatclubandresort</t>
+          <t>facebook.com/rangadip.rangamati</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Family suite Tk 16,000; 1N2D lake package Tk 10,000 (pick-up, kayak, breakfast)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Capacity not found</t>
+          <t>Listed on Agoda, Trip.com, Hotels.com</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Phones conflict</t>
+          <t>Exists; 2 websites</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Nilanjana%20Boat%20Club%20and%20Resort%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rangadip%20Resort%20Rangamati</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>avijatrik.org; tripbangla; offerong</t>
+          <t>facebook; agoda h81757939</t>
         </is>
       </c>
     </row>
@@ -984,67 +984,67 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Bargee Lake Valley (+ Camping)</t>
+          <t>Nilanjana Boat Club &amp; Resort</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Budget eco-resort</t>
+          <t>Floating + hilltop cottages</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Boradam / Manikchori Mukh, Asambosti-Kaptai Rd</t>
+          <t>Asambosti, Kaptai Lake (10 min from Tabalchari ghat, 5 min from Hanging Bridge)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Dellye Bagan, Manikchori Mukh, Boradam, Rangamati Sadar 4500</t>
+          <t>Asham Bosti, Kaptai Lake, Rangamati</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>No own number found (only Take A Boat platform +880 9601-621641)</t>
+          <t>01833-334311; 01911-060900 (also listed for Shukher Tori houseboat) - CONFLICT</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>info@takeaboat.com (platform, not resort)</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>nilanjanaboatclubresort.reservehotel.net</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/p/Bargee-Lake-Valley-100068030345250 ; facebook.com/p/Bargee-Lake-Valley-Camping-Rangamati-100075681652008</t>
+          <t>facebook.com/nilanjanaboatclubandresort</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Budget; not found</t>
+          <t>Family suite Tk 16,000; 1N2D lake package Tk 10,000 (pick-up, kayak, breakfast)</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Water rides; capacity not found</t>
+          <t>2 floating cottages + hilltop cottages; capacity not found</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Contact via Facebook</t>
+          <t>Phones conflict</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Nilanjana%20Boat%20Club%20and%20Resort%20Rangamati</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>amarlodge.com; takeaboat.com; adarbepari; trippainter</t>
+          <t>avijatrik; offerong; tripbangla</t>
         </is>
       </c>
     </row>
@@ -1054,67 +1054,67 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Aronnak (Aronnok) Holiday Resort</t>
+          <t>Bargee Lake Valley (+ Camping)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Lakeside cottages (Army-run)</t>
+          <t>Eco-resort, camping, houseboat</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Near Circuit House / Infantry Brigade, Rangamati Sadar</t>
+          <t>Boradam / Manikchori Mukh, Asambosti-Kaptai Rd</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Near Infantry Brigade, Rangamati Sadar</t>
+          <t>Dellye Bagan, Manikchori Mukh, Boradam, Rangamati Sadar 4500</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>01769-312021; 01669-312022</t>
+          <t>No own number found (Take A Boat platform +880 9601-621641)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>arannokhtj45@gmail.com</t>
+          <t>info@takeaboat.com (platform)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>parjatanbd.com hotel id 404</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/AronnakHolidayCottage ; facebook.com/aronnok.mk</t>
+          <t>facebook.com/p/Bargee-Lake-Valley-100068030345250 ; ...Camping-Rangamati-100075681652008</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Tk 5,000-10,000/night</t>
+          <t>Rooms Tk 6,000-10,000; houseboat stay ~Tk 2,000 (blog title)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>~4 VIP + 7 ordinary rooms (small for 30 - may need 2 places)</t>
+          <t>Water rides, camping, houseboats</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Consistent across sources</t>
+          <t>No resort phone - use Facebook</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor d7928494; bdbooking; mawbiz</t>
+          <t>amarlodge; takeaboat; adarbepari; trippainter; YouTube QktBTfqbYA8</t>
         </is>
       </c>
     </row>
@@ -1124,67 +1124,67 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Nisarga Pod House / Nisarga River Valley</t>
+          <t>Aronnak (Aronnok) Holiday Resort (Army-run)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Pod cottages, glamping</t>
+          <t>Lakeside cottages</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Shilchori, Kaptai (Karnaphuli bank)</t>
+          <t>Near Infantry Brigade / Circuit House, Rangamati Sadar</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Shilchori, Kaptai upazila</t>
+          <t>Near Infantry Brigade, Rangamati Sadar</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>+880 1829-806801; +880 1818-441100; +880 1628-378633</t>
+          <t>01769-312021; 01669-312022</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>arannokhtj45@gmail.com</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>nisargapodhouse.com</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/p/Nisarga-Pod-House-Kaptai-100063674163695 ; facebook.com/p/Nisarga-River-Valley-Pod-House-Kaptai-100083223187517</t>
+          <t>facebook.com/AronnakHolidayCottage ; facebook.com/aronnok.mk</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Tk 5,000/2 people incl. meals + kayak; Tk 6,000/3 people</t>
+          <t>Tk 5,000-10,000/night (~11,490 non-military); boating Tk 600/hr</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Capacity not found; barbecue, kayaking; Dhaka Tribune feature</t>
+          <t>~4 VIP + 7 ordinary rooms - too small alone for 30</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Multiple numbers - confirm</t>
+          <t>Consistent</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Nisarga%20Pod%20House%20Kaptai</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>dhakatribune.com; trip.com; nisargapodhouse.com</t>
+          <t>parjatanbd id 404; tripadvisor d7928494; bdbooking</t>
         </is>
       </c>
     </row>
@@ -1194,27 +1194,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Eco Valley</t>
+          <t>Nisarga Pod House / River Valley</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Camping, bamboo cottages</t>
+          <t>Pod cottages, glamping</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Near Kaptai Lake, Rangamati</t>
+          <t>Shilchori / Rajasthali area, Kaptai (Karnaphuli bank)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Not found (see website)</t>
+          <t>Shilchori, Kaptai upazila</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not found (FB post mentions WhatsApp)</t>
+          <t>+880 1829-806801; +880 1818-441100; +880 1628-378633 (booking 9am-10pm)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1224,37 +1224,37 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>kaptaiecovalley.com</t>
+          <t>nisargapodhouse.com</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/KaptaiEcoValley</t>
+          <t>facebook.com/p/Nisarga-Pod-House-Kaptai-100063674163695 ; ...Nisarga-River-Valley-Pod-House-Kaptai-100083223187517</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>From Tk 1,200/night</t>
+          <t>Tk 5,000 for 2 (meals + kayak); Tk 6,000 for 3</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Tents/cottages, bonfire, kayaking - good for large groups</t>
+          <t>Barbecue, kayaking; capacity not found</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Phone missing</t>
+          <t>Multiple numbers</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Eco%20Valley</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Nisarga%20Pod%20House%20Kaptai</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>kaptaiecovalley.com; tourfo.com</t>
+          <t>dhakatribune; trip.com; hotels.com</t>
         </is>
       </c>
     </row>
@@ -1264,27 +1264,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Riverview Camping Point (KRCP)</t>
+          <t>Kaptai Eco Valley</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Camping</t>
+          <t>Camping, bamboo cottages</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Kaptaimukh, opposite Kaptai Union Parishad Office</t>
+          <t>Near Kaptai Lake, Rangamati</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Kaptaimukh, Kaptai</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>+880 1795-166199; +880 1816-110300</t>
+          <t>Not found (see website/tourfo.com)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1294,37 +1294,37 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>kaptaiecovalley.com (/packages)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/KCP1BD</t>
+          <t>facebook.com/KaptaiEcoValley</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>From Tk 1,200/person/night; 5% weekday discount</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Camping - possible for big group</t>
+          <t>Tents/cottages, tribal dining, bonfire, kayaking - good for large groups</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>FB snippet only</t>
+          <t>Phone missing</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Riverview%20Camping%20Point%20Kaptaimukh</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Eco%20Valley</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/KCP1BD</t>
+          <t>kaptaiecovalley.com; tourfo.com</t>
         </is>
       </c>
     </row>
@@ -1334,27 +1334,27 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Lake Paradise Picnic Spot &amp; Resort</t>
+          <t>Kaptai Riverview Camping Point (KRCP)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Picnic spot + cottages (Navy-linked page)</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Kaptai</t>
+          <t>Kaptaimukh, opp. Kaptai Union Parishad Office</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Kaptaimukh, Kaptai</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1795-166199; +880 1816-110300</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1364,12 +1364,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>lakeparadisebd.com</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/NavyPicnicSpotKaptai</t>
+          <t>facebook.com/KCP1BD ; facebook.com/river.view175</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1379,22 +1379,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Lake/hill-view cottage rooms</t>
+          <t>Camping</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>No contact found</t>
+          <t>FB snippet</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20Paradise%20Kaptai</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Riverview%20Camping%20Point%20Kaptaimukh</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>lakeparadisebd.com</t>
+          <t>facebook</t>
         </is>
       </c>
     </row>
@@ -1404,27 +1404,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Green River View Hotel / Guest House</t>
+          <t>Lake Paradise Picnic Spot &amp; Resort (Navy)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Guest house</t>
+          <t>Picnic spot + 2 cottages</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Kaptaimukh, Kaptai</t>
+          <t>Navy Rd, Kaptai</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Kaptaimukh, Chattogram</t>
+          <t>Navy Rd, Kaptai</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>01889-777830; 01819-351050</t>
+          <t>01769-772174; 01828-915543 - CONFLICT</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1434,37 +1434,37 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>lakeparadisebd.com</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/greenriverviewkaptaihotel</t>
+          <t>facebook.com/NavyPicnicSpotKaptai</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>~Tk 6,000+/night (one review)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Lake/hill view</t>
+          <t>2 cottages x 2 rooms; overnight may need Navy/Army recommendation - NOT suitable for 30</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>From Bangla snippet</t>
+          <t>Restricted</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Green%20River%20View%20Kaptai%20Hotel</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20Paradise%20Kaptai</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>vromontrips/vromonguide snippet; FB</t>
+          <t>asiafirms d427221; lakeparadisebd.com</t>
         </is>
       </c>
     </row>
@@ -1474,42 +1474,42 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Polwel Park &amp; Cottage</t>
+          <t>Green River View Hotel / Guest House</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Resort (run by Rangamati District Police)</t>
+          <t>Guest house</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>DC Bungalow Road, Rangamati</t>
+          <t>Upstream Jetty Ghat, Kaptaimukh</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>DC Bungalow Road, Rangamati</t>
+          <t>56 No. Upstream Jetty Ghat, Kaptai</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>01877-725541; 01877-725542</t>
+          <t>01889-777830; 01819-351050</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>polwelresort@gmail.com</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>polwelpark.com</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/greenriverviewkaptaihotel</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -1519,22 +1519,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Luxury, secured</t>
+          <t>Lake/hill view</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Snippet only</t>
+          <t>Reported open</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20and%20Cottage%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Green%20River%20View%20Kaptai%20Hotel</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>tripsilo; vromonguide snippet</t>
+          <t>facebook; vromonguide</t>
         </is>
       </c>
     </row>
@@ -1544,27 +1544,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Parjatan Holiday Complex Rangamati</t>
+          <t>Hotel Happiness Hill</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Govt (BPC) hotel</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Hanging Bridge Road, Rangamati town</t>
+          <t>Upstream Jetty Ghat, Kaptai</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Hanging Bridge Rd, Rangamati Sadar</t>
+          <t>27 No. Upstream Jetty Ghat, Kaptai, Rangamati</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>02-333371853 / 02-333371851; 01863-231185; 01991-139037; 0351-63126</t>
+          <t>01970-329335; 01752-328837</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1574,37 +1574,37 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/hotelhappinesshill</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Tk 1,600-6,000/night</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Easiest official group booking</t>
+          <t>On Agoda</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Bangla snippet</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Happiness%20Hill%20Kaptai</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>hotels.gov.bd; tripadvisor</t>
+          <t>agoda; vromontrips/goofly24 snippet</t>
         </is>
       </c>
     </row>
@@ -1614,67 +1614,67 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Hotel Jum Palace</t>
+          <t>Rainya Tugun (Raina Togun) Eco Resort</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Eco resort</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Opp. post office, T&amp;T Area, Rangamati</t>
+          <t>Kamilachari, Mogban, Rangamati Sadar (15 km from town)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>T&amp;T Area, Rangamati</t>
+          <t>Vill Kamilachari, Union Mogban, Rangamati Sadar</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>0351-61878; 01625-100000</t>
+          <t>01551-708244; 01781-136071</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>See website</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>jumpalace.com</t>
+          <t>rainyatugun.com</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>facebook.com/HotelJumPalacebd</t>
+          <t>facebook.com/rainyatugunecoresort ; facebook.com/rainyatugun</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Tk 1,500-3,200/night</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Eco resort</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Consistent</t>
+          <t>Exists</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rainya%20Tugun%20Eco%20Resort%20Rangamati</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>jumpalace.com; snippets</t>
+          <t>rainyatugun.com; tourtoday.com.bd</t>
         </is>
       </c>
     </row>
@@ -1684,22 +1684,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Hotel Shanghai International</t>
+          <t>Borgang Eco Cottage (Kaptai Lakeside Eco Cottage)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Community eco cottage</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Central Rangamati</t>
+          <t>Borgang, ~13 km from Rangamati town</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Rangamati town</t>
+          <t>Borgang, Rangamati</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1729,22 +1729,22 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>28 rooms, free breakfast</t>
+          <t>Cottages (Bijhu/Boishu/Shangrai), tribal restaurant, boats</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>No contact found</t>
+          <t>Contact via avijatrik</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Borgang%20Eco%20Cottage%20Rangamati</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor d10348460</t>
+          <t>avijatrik.org/tour/borgang-eco-cottage-rangamati</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Rangadip / Ranga Dwip Resort</t>
+          <t>Rreng Lake Beach Resort &amp; Restaurant</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1764,17 +1764,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Rangamati</t>
+          <t>Morghona / Boradam, Rangamati</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Boradam, Rangamati</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not found (FB says 'call')</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/p/Rreng-Lake-beach-Resort-Restaurant-61568391382920</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1799,22 +1799,22 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Unverified</t>
+          <t>Lakeside</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Unverified name</t>
+          <t>Contact via FB</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rangadip%20Resort%20Rangamati</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rreng%20Lake%20Beach%20Resort%20Rangamati</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>tripadvisor listing mention</t>
+          <t>facebook</t>
         </is>
       </c>
     </row>
@@ -1824,22 +1824,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Raina Togun Eco Resort</t>
+          <t>Gang Sabarang</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Eco resort</t>
+          <t>Lakeside restaurant + cottages, kayak</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Kaptai</t>
+          <t>Assambasti, Rangamati</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Assambasti, Rangamati</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/gangsabarang</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1869,22 +1869,22 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Bangla snippet only</t>
+          <t>Cottage rental</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>UNVERIFIED - follow-up search found nothing</t>
+          <t>Contact via FB</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Raina%20Togun%20Eco%20Resort%20Kaptai</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Gang%20Sabarang%20Rangamati</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>goofly24/vromonguide snippet</t>
+          <t>tripadvisor d15141023</t>
         </is>
       </c>
     </row>
@@ -1894,67 +1894,837 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
+          <t>Polwel Park &amp; Cottage (Police-run)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Resort/park</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>DC Bungalow Road, Rangamati</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>DC Bungalow Road, Rangamati</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>+880 1877-725541; 01877-725542; ticket 01877-725540</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>polwelpark@gmail.com (also polwelresort@gmail.com reported)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>polwelpark.com</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/PolwelParkRmtOfficialPage</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Luxury, secured</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>polwelpark.com; tripsilo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Parjatan Holiday Complex Rangamati</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Govt (BPC) hotel</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Hanging Bridge Road, Rangamati town</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Hanging Bridge Rd, Rangamati Sadar</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>01863-231185; 01991-139037; 02-333371853 / 02-333371851 (head-office style); 0351-63126</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>contact@parjatan.gov.bd</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Non-AC twin Tk 900; AC twin 1,900; tribal cottage 1,300; full cottage 2,500</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Breakfast included; official group booking</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Consistent</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>hotels.gov.bd; parjatanbd id 816; wikimapia 17123711</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Jum Palace</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Opp. post office, T&amp;T Area, Rangamati</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>T&amp;T Area, Rangamati</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>0351-61878; 01625-100000</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>booking@jumpalace.com</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>jumpalace.com</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/HotelJumPalacebd</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Tk 1,500-3,200</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Consistent</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>jumpalace.com; parjatanbd id 401</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Shanghai International</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Hotel (28 rooms)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Chandraghona Rd / Kathaltali, Rangamati</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Kathaltali, Chandraghona Road, Rangamati</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>0351-61402; 01730-195778; 01740-988532; 01820-309000</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/hotelshanghaiintrangamati</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Tk 1,000-3,000 (2-bed 2,000; 3-bed 2,000; couple non-AC 1,500)</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Free breakfast; 28 rooms</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>tour.com.bd; bdbooking; findglocal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
           <t>Hotel Rajmahal International</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar, Rangamati (address contradictory)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar / near Parjatan area</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>01819-508628</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>reservation@rajmahalinternational.com (low confidence)</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>rajmahal.hotelsofbangladesh.com</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/HotelRajmahal.int</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Low confidence</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Rajmahal%20International%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>facebook; amarlodge</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Hill City</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar, Rangamati</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>01828-819326</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Snippet only</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20City%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>vromonguide snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Hill</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar, Rangamati</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Reserve Bazar</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>0351-62843; 01866-609400</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Snippet only</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>vromonguide snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Forest Dept Rest House</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Govt rest house</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Banarupa, Rangamati</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Banarupa</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>0351-63351</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Govt booking</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Snippet only</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Forest%20Rest%20House%20Banarupa%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>vromonguide snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Sonar Bangla</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Seen, not researched</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>sonar-bangla.bangladeshhotels.net</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>~US$18-33</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Listing only</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sonar%20Bangla%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>bangladeshhotels.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Green Castle</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati / Kaptai (unclear)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>01859-778065 (same as Lakeshore - doubtful)</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>green-castle.bangladeshhotels.net</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>~US$12; Tk 600-2,500</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Budget hotel</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Doubtful</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Green%20Castle%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>bangladeshhotels.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Zoomking Eco Resort / Izor Resort / Berainnya Resort</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Resorts (names only)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Kaptai Lake</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Names from resortian.com only; Prothom Alo: ~20 resorts on lake, only 3 with environmental clearance</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Rajmahal%20International%20Rangamati</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>search snippet</t>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Zoomking%20Eco%20Resort%20Kaptai</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>resortian (snippet); prothomalo b5frd0vwuj</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Hotel Sufia / Moti Mahal / Hotel Prince</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Hotels (names only)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Rangamati</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Names from vromonguide snippet only</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sufia%20Rangamati</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>vromonguide snippet</t>
         </is>
       </c>
     </row>
@@ -1980,6 +2750,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1991,16 +2772,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -2022,12 +2803,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Phone / WhatsApp</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Website / Source</t>
+          <t>Website / Email</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2059,17 +2840,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Lake, Rangamati</t>
+          <t>Kaptai Lake</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>+880 1711-336825; 01402-288573; 01678-076361; 01911-060900 (also Nilanjana's - verify)</t>
+          <t>Not found (older reports: +880 1711-336825; 01402-288573; 01911-060900 - unverified)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>bdcruise.com/royal-adventure/ ; hoihullorholidays.com/royal-adventure/</t>
+          <t>bdcruise.com/royal-adventure ; takeaboat.com ; hoihullorholidays.com/royal-adventure</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -2079,29 +2860,29 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>8 rooms x 4 = up to 32 people; 2D1N package; price Tk 85,000 (6 ppl) - 115,000 (12 ppl) per source</t>
+          <t>8 rooms x 4 = ~32 people (UNB, Prothom Alo); price for 30 not found</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Best houseboat fit for 30</t>
+          <t>BEST houseboat fit for 30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Promodini Boat Life (Avijatrik Tourism)</t>
+          <t>Promodini Boat Life</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Houseboat x2</t>
+          <t>Houseboats</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Kaptai Lake, Rangamati</t>
+          <t>Kaptai Lake</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2111,96 +2892,96 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>avijatrik.org/tour/promodini-boat-life</t>
+          <t>bdcruise.com/kaptai-promodini ; avijatrik.org/tour/promodini-boat-life</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/PromodiniBoatLife</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Promodini-1 sleeps 6 + Promodini-2 sleeps 10 = 16 only</t>
+          <t>6-12 per boat, so 30 needs 3+ boats; snippets: Tk 6,000/person; Tk 85,000 (6)-115,000 (12) unverified</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Too small alone for 30</t>
+          <t>2D1N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BD Cruise</t>
+          <t>Shukher (Sukher) Tori</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Tour operator/houseboats</t>
+          <t>Houseboat</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Rangamati-Kaptai</t>
+          <t>Kaptai Lake</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>01911-060900</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>bdcruise.com/rangamati-kaptai-lake/</t>
+          <t>hoihullorholidays.com/shukher-tori</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/sukhertorihouseboat</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Tk 8,000 for 2D1N (per source); 6 AC cabins</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Ask for 30-person quote</t>
+          <t>Small - would need multiple</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GoZayaan</t>
+          <t>Rangatori (রাঙ্গাতরী)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tour operator</t>
+          <t>Houseboat</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Kaptai Lake, Rangamati</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 1853-496162 (WhatsApp wa.me/8801853496162); +880 1828-907706</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>gozayaan.com/destination/rangamati-tour-package</t>
+          <t>rangatori.rgt@gmail.com</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>facebook.com/rangatori.rgt</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -2210,24 +2991,24 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Package quote</t>
+          <t>Contact for 30-person quote</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Galaxy Holidays BD</t>
+          <t>BD Cruise</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Tour operator</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Rangamati-Kaptai</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2237,7 +3018,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>galaxyholidaysbd.com/package/Rangamati-Chittagong</t>
+          <t>bdcruise.com/rangamati-kaptai-lake</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2252,19 +3033,19 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Package quote</t>
+          <t>Ask quote</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ITS Holidays Ltd</t>
+          <t>Take A Boat (platform)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Tour operator</t>
+          <t>Booking platform</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2274,12 +3055,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>+880 9601-621641</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>itsholidaysltd.com/rangamati-and-kaptai-tour-package</t>
+          <t>takeaboat.com ; info@takeaboat.com</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2294,19 +3075,19 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Package quote</t>
+          <t>Lists Bargee, Royal Adventure</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Bangladesh Travel and Tours / Hoihullor Holidays</t>
+          <t>GoZayaan</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tour operators</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2321,7 +3102,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>bangladeshtravelandtours.com ; hoihullorholidays.com</t>
+          <t>gozayaan.com/destination/rangamati-tour-package</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2336,49 +3117,259 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Houseboat packages</t>
+          <t>Quote</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>General Rangamati hotel &amp; boat booking line</t>
+          <t>Galaxy Holidays BD</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Unverified number</t>
+          <t>Operator</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>galaxyholidaysbd.com/package/Rangamati-Chittagong</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ITS Holidays Ltd</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>itsholidaysltd.com/rangamati-and-kaptai-tour-package</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Avijatrik Tourism</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Operator (Promodini, Borgang, Divine)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>avijatrik.org</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Bangladesh Travel &amp; Tours / Hoihullor Holidays</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Operators</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>bangladeshtravelandtours.com ; hoihullorholidays.com</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Lake boat hire (ghats: Parjatan, Banarupa, Reserve Bazar)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Local boats</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>+880 1841-862600 (single Bangla snippet)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>No operator numbers</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>tbsnews.net three-popular-places-visit-rangamati</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Engine boat Tk 1,000-2,500 (10-15 people); speedboat ~Tk 1,200-1,500/hr; Aronnak boating Tk 600/hr</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Need 2-3 boats for 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka coach hire (reference)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Bus rental</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Dhaka</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>minibusbd.com ; travelmate.com.bd ; hotel.com.bd</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Unverified</t>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>30-seat AC bus ~Tk 23,000/day (DHAKA CITY rate, not to Rangamati); Dhaka-Rangamati ~304 km, 7-9 hrs</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Get intercity quote</t>
         </is>
       </c>
     </row>
@@ -2393,65 +3384,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="130" customWidth="1" min="1" max="1"/>
+    <col width="140" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Research log (autoresearch-style loop: metric = distinct resorts found; keep new/verified, discard duplicates)</t>
+          <t>Research log (autoresearch-style loop; metric = distinct places with verified contacts)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Round 1 (single search): 12 entries. Round 2 (4 parallel agents: Facebook/social, YouTube/blogs, verification, Kaptai-upazila): 19 stay entries + 8 houseboat/operator entries after de-duplication.</t>
+          <t>Round 1: 12 entries. Round 2: 4 agents -&gt; 19 stays + 8 operators. Round 3: 4 agents (gap-fill x2, discovery, operators) -&gt; 31 rows here (some rows group several unverified names) + 13 boat/transport rows.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>LIMITS: Facebook, YouTube, Instagram, X, TripAdvisor and most Bangla travel blogs were blocked from this environment (proxy); only search-result snippets were readable. YouTube/X gave nothing usable.</t>
+          <t>HARD LIMIT: Facebook, YouTube, Instagram, X, TripAdvisor, and nearly every travel blog/operator website were blocked from this environment. All data is from search-result snippets, not the pages themselves. YouTube/X yielded nothing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>No coordinates or exact Google Maps place URLs found; the Maps links are name searches - confirm the pin.</t>
+          <t>Still 'Not found' after 3 rounds: WhatsApp numbers (except Rangatori), latitude/longitude, exact Google Maps place URLs, day-picnic/meal prices, most emails, Kaptai Eco Valley phone, Bargee's own phone, and operator phones for BD Cruise/GoZayaan/Galaxy/ITS/Avijatrik.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Phones conflict for Lakeshore, Lake View Island, Divine Lake Island, Nilanjana; Hill Taj number may be a payment number; Bargee has only a platform number. CALL AND CONFIRM before advance payment.</t>
+          <t>Phones conflict for Lakeshore, Lake View Island, Divine Lake Island, Hill Taj, Nilanjana, Lake Paradise; 01911-060900 appears for both Nilanjana and Shukher Tori. Call and confirm before any advance payment.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Prices are old blog/listing figures. Ask for 30-person group rate, meals, boat transfer, whole-resort booking.</t>
+          <t>Google Maps links are name searches (no pin coordinates found) - verify the pin.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Not opened (blocked; try on your own network): vromonguide.com/hotels-and-resorts-in-rangamati, bd-info.com/rangamati-hotel-resort-list, ratekom.com list, goofly24 blog, resortian.com/blog/kaptai-lake-resorts, TripAdvisor hotels near Kaptai Lake.</t>
+          <t>Prothom Alo reports ~20 resorts around the lake and only 3 with environmental clearance - ask about legal/permit status.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Shortlist for 30 people: Lakeshore (whole-resort), Royal Adventure houseboat (32 cap.), Kaptai Eco Valley (camping), Parjatan Holiday Complex (official), or split between Aronnak + another.</t>
+          <t>Some resorts are Army/Navy/Police-run; civilian overnight access may need permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Pages worth opening on your own network to fill the gaps: vromonguide.com/hotels-and-resorts-in-rangamati, bd-info.com/rangamati-hotel-resort-list, ratekom.com list, goofly24 Kaptai list, travelvibe.net/rangamati-hotels-list, resortian.com/blog/kaptai-lake-resorts, each resort's Facebook About page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Shortlist for 30: Lakeshore (whole resort) ; Royal Adventure houseboat (32 cap.) ; Kaptai Eco Valley (camping) ; Parjatan Holiday Complex ; or split groups across e.g. Aronnak + Divine Lake Island / Wildwood.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add photo search link column beside each resort
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164MYEZuLZ1BUVpVHt4sH1c
</commit_message>
<xml_diff>
--- a/Kaptai_Rangamati_Resorts.xlsx
+++ b/Kaptai_Rangamati_Resorts.xlsx
@@ -467,23 +467,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,60 +500,65 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Photos (click - Google Images)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Phone / Booking</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Facebook / Social</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Capacity / Notes for 30</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Verification</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Google Maps (search link)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
@@ -567,62 +573,67 @@
           <t>Lakeshore Resort, Kaptai</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Lakeshore%20Resort%2C%20Kaptai%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Lakeside resort</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Kaptaimukh / Jeebtoli, Kaptai</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Jeebtali-Log Gate Link Road, Kaptaimukh, Kaptai, Chattogram 4530</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>01859-778065 (most cited); 01550-322448 (asiafirms) - CONFLICT</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Obfuscated in sources</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>aronnok.com may be sister property (Aronnok &amp; Lakeshore)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>facebook.com/LakeshoreResortKaptai</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Room ~Tk 5,000 (range 4,500-9,000); WHOLE RESORT ~Tk 40,000/night; kayak Tk 200/hr; entry Tk 50</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>15 cottages, AC rooms, pool, restaurant/BBQ, 200ft hanging bridge; whole-resort booking - BEST FIT for 30</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Multi-source; phones conflict</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lakeshore%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>hotelresortbd.com; asiafirms; marketbangladesh; tourtobangladesh; tripbangla</t>
         </is>
@@ -637,31 +648,31 @@
           <t>Lake View Island Resort (Army-run)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Lake%20View%20Island%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Island resort</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Island ~10 min boat from Kaptai ghat</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Kaptai Lake, Kaptai (boat access)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>01769-322183; 01769-322182; 01746-191421 / 01847-191421; 0179322172/3 (malformed) - CONFLICT</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -669,30 +680,35 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/kaptai.island2016 ; facebook.com/p/Lakeview-Island-Resort-100086979506274</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Civilian Tk 4,300/room/night; military Tk 1,025; 25% advance</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Cottages, restaurant, houseboat, boat club; cottage count not found</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20View%20Island%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>lrbtravelteam; tripadvisor d13974943; vromonguide</t>
         </is>
@@ -707,62 +723,67 @@
           <t>Divine Lake Island Resort</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Divine%20Lake%20Island%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Island resort (6 acre)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Near Asambosti bridge, Kaptai Road</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Kaptai Road, Ashambosti, Rangamati 4500 (call reception at Asambosti pier; free shuttle boat ~30 min)</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>01611-585887 (2 sources); 01958-054408 (1 source)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>divinelakeisland.com</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>facebook.com/divinelakeisland</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>AC cottage Tk 6,000; bamboo cottage Tk 4,000-4,500</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>2 AC + 4 bamboo cottages (packages 2-15 people) - too small alone for 30</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Ashambosti%20Rangamati</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>avijatrik; tripsilo; booking.com</t>
         </is>
@@ -777,62 +798,67 @@
           <t>Hill Taj Resort / The Grand Hill Taj</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hill%20Taj%20Resort%20/%20The%20Grand%20Hill%20Taj%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Island resort + water park</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Kaptai Lake, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Kaptai Lake, Rangamati Sadar 4500; C.O. Office Ghat / Furfura Tila</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>+880 1600-343694; +880 1777-714621 (booking, per bd-info); +880 1870-701892 (merchant/payment?)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>thegrandhilltaj.com</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>facebook.com/thegrandhilltaj</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>OTA from ~US$74; 50% advance; free breakfast; free boat from city</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Treehouse, pool, 24/7 room dining; room count not found</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Numbers conflict</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=The%20Grand%20Hill%20Taj%20Rangamati</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>bd-info; bdbooking; lrbtravelteam; thegrandhilltaj.com</t>
         </is>
@@ -847,62 +873,67 @@
           <t>Wildwood Island Resort</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Wildwood%20Island%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Luxury island resort</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Diglibagh, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Diglibagh, Rangamati 4500</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>+880 1833-334309</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>wildwoodislandresort@gmail.com</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>wildwoodisland.com</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>facebook.com/Wildwoodislandresort</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>~Tk 10,800-12,000/night (reviews); ~US$101 OTA</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Villas: Luxury (Hill View), Superior, Junior, Family; count not found</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>One source per contact</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Wildwood%20Island%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>insidebangla; tripadvisor d33959189; agoda</t>
         </is>
@@ -917,62 +948,67 @@
           <t>Rangadip Resort</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Rangadip%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Private island resort</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
           <t>+880 1327-475252; 01977-792001 (fragment)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>rangadipresort@gmail.com</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>rangadipresort.com / rangadip.com</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>facebook.com/rangadip.rangamati</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
           <t>Listed on Agoda, Trip.com, Hotels.com</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Exists; 2 websites</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rangadip%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>facebook; agoda h81757939</t>
         </is>
@@ -987,62 +1023,67 @@
           <t>Nilanjana Boat Club &amp; Resort</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Nilanjana%20Boat%20Club%20%26%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Floating + hilltop cottages</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Asambosti, Kaptai Lake (10 min from Tabalchari ghat, 5 min from Hanging Bridge)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Asham Bosti, Kaptai Lake, Rangamati</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>01833-334311; 01911-060900 (also listed for Shukher Tori houseboat) - CONFLICT</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>nilanjanaboatclubresort.reservehotel.net</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>facebook.com/nilanjanaboatclubandresort</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Family suite Tk 16,000; 1N2D lake package Tk 10,000 (pick-up, kayak, breakfast)</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>2 floating cottages + hilltop cottages; capacity not found</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Nilanjana%20Boat%20Club%20and%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>avijatrik; offerong; tripbangla</t>
         </is>
@@ -1057,62 +1098,67 @@
           <t>Bargee Lake Valley (+ Camping)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Bargee%20Lake%20Valley%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Eco-resort, camping, houseboat</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Boradam / Manikchori Mukh, Asambosti-Kaptai Rd</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Dellye Bagan, Manikchori Mukh, Boradam, Rangamati Sadar 4500</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>No own number found (Take A Boat platform +880 9601-621641)</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>info@takeaboat.com (platform)</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/p/Bargee-Lake-Valley-100068030345250 ; ...Camping-Rangamati-100075681652008</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Rooms Tk 6,000-10,000; houseboat stay ~Tk 2,000 (blog title)</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Water rides, camping, houseboats</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>No resort phone - use Facebook</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t>amarlodge; takeaboat; adarbepari; trippainter; YouTube QktBTfqbYA8</t>
         </is>
@@ -1127,62 +1173,67 @@
           <t>Aronnak (Aronnok) Holiday Resort (Army-run)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Aronnak%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Lakeside cottages</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Near Infantry Brigade / Circuit House, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Near Infantry Brigade, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>01769-312021; 01669-312022</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>arannokhtj45@gmail.com</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/AronnakHolidayCottage ; facebook.com/aronnok.mk</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Tk 5,000-10,000/night (~11,490 non-military); boating Tk 600/hr</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>~4 VIP + 7 ordinary rooms - too small alone for 30</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Consistent</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>parjatanbd id 404; tripadvisor d7928494; bdbooking</t>
         </is>
@@ -1197,62 +1248,67 @@
           <t>Nisarga Pod House / River Valley</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Nisarga%20Pod%20House%20/%20River%20Valley%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Pod cottages, glamping</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Shilchori / Rajasthali area, Kaptai (Karnaphuli bank)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Shilchori, Kaptai upazila</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>+880 1829-806801; +880 1818-441100; +880 1628-378633 (booking 9am-10pm)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
           <t>nisargapodhouse.com</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>facebook.com/p/Nisarga-Pod-House-Kaptai-100063674163695 ; ...Nisarga-River-Valley-Pod-House-Kaptai-100083223187517</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Tk 5,000 for 2 (meals + kayak); Tk 6,000 for 3</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Barbecue, kayaking; capacity not found</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Multiple numbers</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Nisarga%20Pod%20House%20Kaptai</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t>dhakatribune; trip.com; hotels.com</t>
         </is>
@@ -1267,62 +1323,67 @@
           <t>Kaptai Eco Valley</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Kaptai%20Eco%20Valley%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Camping, bamboo cottages</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Near Kaptai Lake, Rangamati</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>Not found (see website/tourfo.com)</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
           <t>kaptaiecovalley.com (/packages)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>facebook.com/KaptaiEcoValley</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>From Tk 1,200/person/night; 5% weekday discount</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Tents/cottages, tribal dining, bonfire, kayaking - good for large groups</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Phone missing</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Eco%20Valley</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>kaptaiecovalley.com; tourfo.com</t>
         </is>
@@ -1337,31 +1398,31 @@
           <t>Kaptai Riverview Camping Point (KRCP)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Kaptai%20Riverview%20Camping%20Point%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Camping</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Kaptaimukh, opp. Kaptai Union Parishad Office</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Kaptaimukh, Kaptai</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>+880 1795-166199; +880 1816-110300</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1369,30 +1430,35 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/KCP1BD ; facebook.com/river.view175</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
           <t>Camping</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>FB snippet</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="N13" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Riverview%20Camping%20Point%20Kaptaimukh</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="O13" s="2" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
@@ -1407,62 +1473,67 @@
           <t>Lake Paradise Picnic Spot &amp; Resort (Navy)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Lake%20Paradise%20Picnic%20Spot%20%26%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Picnic spot + 2 cottages</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Navy Rd, Kaptai</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Navy Rd, Kaptai</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>01769-772174; 01828-915543 - CONFLICT</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
           <t>lakeparadisebd.com</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>facebook.com/NavyPicnicSpotKaptai</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>~Tk 6,000+/night (one review)</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>2 cottages x 2 rooms; overnight may need Navy/Army recommendation - NOT suitable for 30</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Restricted</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20Paradise%20Kaptai</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>asiafirms d427221; lakeparadisebd.com</t>
         </is>
@@ -1477,31 +1548,31 @@
           <t>Green River View Hotel / Guest House</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Green%20River%20View%20Hotel%20/%20Guest%20House%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Guest house</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Upstream Jetty Ghat, Kaptaimukh</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>56 No. Upstream Jetty Ghat, Kaptai</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>01889-777830; 01819-351050</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1509,30 +1580,35 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/greenriverviewkaptaihotel</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
           <t>Lake/hill view</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Reported open</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Green%20River%20View%20Kaptai%20Hotel</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>facebook; vromonguide</t>
         </is>
@@ -1547,31 +1623,31 @@
           <t>Hotel Happiness Hill</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Happiness%20Hill%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Upstream Jetty Ghat, Kaptai</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>27 No. Upstream Jetty Ghat, Kaptai, Rangamati</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>01970-329335; 01752-328837</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1579,30 +1655,35 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/hotelhappinesshill</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
           <t>On Agoda</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Bangla snippet</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Happiness%20Hill%20Kaptai</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>agoda; vromontrips/goofly24 snippet</t>
         </is>
@@ -1617,62 +1698,67 @@
           <t>Rainya Tugun (Raina Togun) Eco Resort</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Rainya%20Tugun%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Eco resort</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Kamilachari, Mogban, Rangamati Sadar (15 km from town)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Vill Kamilachari, Union Mogban, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>01551-708244; 01781-136071</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>rainyatugun.com</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>facebook.com/rainyatugunecoresort ; facebook.com/rainyatugun</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
           <t>Eco resort</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rainya%20Tugun%20Eco%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>rainyatugun.com; tourtoday.com.bd</t>
         </is>
@@ -1687,26 +1773,26 @@
           <t>Borgang Eco Cottage (Kaptai Lakeside Eco Cottage)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Borgang%20Eco%20Cottage%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Community eco cottage</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Borgang, ~13 km from Rangamati town</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Borgang, Rangamati</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1729,20 +1815,25 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
           <t>Cottages (Bijhu/Boishu/Shangrai), tribal restaurant, boats</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Contact via avijatrik</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Borgang%20Eco%20Cottage%20Rangamati</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>avijatrik.org/tour/borgang-eco-cottage-rangamati</t>
         </is>
@@ -1757,31 +1848,31 @@
           <t>Rreng Lake Beach Resort &amp; Restaurant</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Rreng%20Lake%20Beach%20Resort%20%26%20Restaurant%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Resort</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Morghona / Boradam, Rangamati</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Boradam, Rangamati</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Not found (FB says 'call')</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1789,30 +1880,35 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/p/Rreng-Lake-beach-Resort-Restaurant-61568391382920</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
           <t>Lakeside</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Contact via FB</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rreng%20Lake%20Beach%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
@@ -1827,26 +1923,26 @@
           <t>Gang Sabarang</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Gang%20Sabarang%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Lakeside restaurant + cottages, kayak</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Assambasti, Rangamati</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Assambasti, Rangamati</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -1859,30 +1955,35 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/gangsabarang</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
           <t>Cottage rental</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Contact via FB</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="N20" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Gang%20Sabarang%20Rangamati</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>tripadvisor d15141023</t>
         </is>
@@ -1897,62 +1998,67 @@
           <t>Polwel Park &amp; Cottage (Police-run)</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Polwel%20Park%20%26%20Cottage%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Resort/park</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>DC Bungalow Road, Rangamati</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>DC Bungalow Road, Rangamati</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>+880 1877-725541; 01877-725542; ticket 01877-725540</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>polwelpark@gmail.com (also polwelresort@gmail.com reported)</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>polwelpark.com</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>facebook.com/PolwelParkRmtOfficialPage</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
           <t>Luxury, secured</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="N21" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20Rangamati</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="O21" s="2" t="inlineStr">
         <is>
           <t>polwelpark.com; tripsilo</t>
         </is>
@@ -1967,62 +2073,67 @@
           <t>Parjatan Holiday Complex Rangamati</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Parjatan%20Holiday%20Complex%20Rangamati%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Govt (BPC) hotel</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Hanging Bridge Road, Rangamati town</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Hanging Bridge Rd, Rangamati Sadar</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>01863-231185; 01991-139037; 02-333371853 / 02-333371851 (head-office style); 0351-63126</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>contact@parjatan.gov.bd</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>hotels.gov.bd/frontend/hotel/15-holiday-complex-rangamati</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
           <t>Non-AC twin Tk 900; AC twin 1,900; tribal cottage 1,300; full cottage 2,500</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Breakfast included; official group booking</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Consistent</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>hotels.gov.bd; parjatanbd id 816; wikimapia 17123711</t>
         </is>
@@ -2037,62 +2148,67 @@
           <t>Hotel Jum Palace</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Jum%20Palace%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Opp. post office, T&amp;T Area, Rangamati</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>T&amp;T Area, Rangamati</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>0351-61878; 01625-100000</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>booking@jumpalace.com</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>jumpalace.com</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>facebook.com/HotelJumPalacebd</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>Tk 1,500-3,200</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Consistent</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>jumpalace.com; parjatanbd id 401</t>
         </is>
@@ -2107,31 +2223,31 @@
           <t>Hotel Shanghai International</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Shanghai%20International%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Hotel (28 rooms)</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Chandraghona Rd / Kathaltali, Rangamati</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Kathaltali, Chandraghona Road, Rangamati</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>0351-61402; 01730-195778; 01740-988532; 01820-309000</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2139,30 +2255,35 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
           <t>facebook.com/hotelshanghaiintrangamati</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Tk 1,000-3,000 (2-bed 2,000; 3-bed 2,000; couple non-AC 1,500)</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>Free breakfast; 28 rooms</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>tour.com.bd; bdbooking; findglocal</t>
         </is>
@@ -2177,62 +2298,67 @@
           <t>Hotel Rajmahal International</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Rajmahal%20International%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar, Rangamati (address contradictory)</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar / near Parjatan area</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>01819-508628</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>reservation@rajmahalinternational.com (low confidence)</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>rajmahal.hotelsofbangladesh.com</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>facebook.com/HotelRajmahal.int</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>Low confidence</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Rajmahal%20International%20Rangamati</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>facebook; amarlodge</t>
         </is>
@@ -2247,31 +2373,31 @@
           <t>Hotel Hill City</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Hill%20City%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar, Rangamati</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>01828-819326</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2289,20 +2415,25 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="N26" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20City%20Rangamati</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2317,31 +2448,31 @@
           <t>Hotel Hill</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Hill%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar, Rangamati</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Reserve Bazar</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>0351-62843; 01866-609400</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2359,20 +2490,25 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="N27" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20Rangamati</t>
         </is>
       </c>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2387,31 +2523,31 @@
           <t>Forest Dept Rest House</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Forest%20Dept%20Rest%20House%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Govt rest house</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Banarupa, Rangamati</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Banarupa</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>0351-63351</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2429,20 +2565,25 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
           <t>Govt booking</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Forest%20Rest%20House%20Banarupa%20Rangamati</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2457,21 +2598,21 @@
           <t>Hotel Sonar Bangla</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Sonar%20Bangla%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2484,35 +2625,40 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
           <t>sonar-bangla.bangladeshhotels.net</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
           <t>~US$18-33</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Listing only</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sonar%20Bangla%20Rangamati</t>
         </is>
       </c>
-      <c r="N29" s="2" t="inlineStr">
+      <c r="O29" s="2" t="inlineStr">
         <is>
           <t>bangladeshhotels.net</t>
         </is>
@@ -2527,62 +2673,67 @@
           <t>Hotel Green Castle</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Green%20Castle%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Rangamati / Kaptai (unclear)</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
           <t>01859-778065 (same as Lakeshore - doubtful)</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
           <t>green-castle.bangladeshhotels.net</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
           <t>~US$12; Tk 600-2,500</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Budget hotel</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Doubtful</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Green%20Castle%20Rangamati</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>bangladeshhotels.net</t>
         </is>
@@ -2597,21 +2748,21 @@
           <t>Zoomking Eco Resort / Izor Resort / Berainnya Resort</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Zoomking%20Eco%20Resort%20/%20Izor%20Resort%20/%20Berainnya%20Resort%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Resorts (names only)</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Kaptai Lake</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2639,20 +2790,25 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
           <t>Names from resortian.com only; Prothom Alo: ~20 resorts on lake, only 3 with environmental clearance</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Zoomking%20Eco%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>resortian (snippet); prothomalo b5frd0vwuj</t>
         </is>
@@ -2667,21 +2823,21 @@
           <t>Hotel Sufia / Moti Mahal / Hotel Prince</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.google.com/search?tbm=isch&amp;q=Hotel%20Sufia%20/%20Moti%20Mahal%20/%20Hotel%20Prince%20Rangamati%20Kaptai</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Hotels (names only)</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Rangamati</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Not found</t>
@@ -2709,20 +2865,25 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
           <t>Names from vromonguide snippet only</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sufia%20Rangamati</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2730,37 +2891,68 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add guest ratings, review pros/cons and group suitability score
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0164MYEZuLZ1BUVpVHt4sH1c
</commit_message>
<xml_diff>
--- a/Kaptai_Rangamati_Resorts.xlsx
+++ b/Kaptai_Rangamati_Resorts.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,10 @@
     <col width="36" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,10 +558,25 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Guest rating (platform, #reviews)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Pros / Cons from reviews &amp; guides</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Suitability for 30 (1-5, my judgement)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Google Maps (search link)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
@@ -628,12 +646,25 @@
           <t>Multi-source; phones conflict</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor 4/5 (17 rev; shared listing 'Aronnok &amp; Lakeshore', #2 of 4 in Rangamati); Facebook 60% recommend (34 rev)</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>+ scenic, peaceful, good food/service; whole-resort option. - pool cleanliness, breakfast</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lakeshore%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>hotelresortbd.com; asiafirms; marketbangladesh; tourtobangladesh; tripbangla</t>
         </is>
@@ -703,12 +734,25 @@
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor: 2 reviews, no score</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>+ scenic, boating, pool, good with friends. - high prices, no AC, hot water issues, poor extra beds, food</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20View%20Island%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>lrbtravelteam; tripadvisor d13974943; vromonguide</t>
         </is>
@@ -778,12 +822,25 @@
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>+ boat pick-up, bamboo/AC cottages, free breakfast (resort's own text). - only 6 cottages; no guest reviews seen</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Divine%20Lake%20Island%20Ashambosti%20Rangamati</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>avijatrik; tripsilo; booking.com</t>
         </is>
@@ -853,12 +910,25 @@
           <t>Numbers conflict</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor 3/5 (#3 of 4 in Rangamati)</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>+ service, staff, playground, pool, free breakfast. - cleanliness/facilities complaints</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=The%20Grand%20Hill%20Taj%20Rangamati</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>bd-info; bdbooking; lrbtravelteam; thegrandhilltaj.com</t>
         </is>
@@ -928,12 +998,25 @@
           <t>One source per contact</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Expedia 4.4/5 (115 rev)</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>+ private island, pool, free breakfast. - one guest called stay 'disappointing'; pricey</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Wildwood%20Island%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>insidebangla; tripadvisor d33959189; agoda</t>
         </is>
@@ -1003,12 +1086,25 @@
           <t>Exists; 2 websites</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Highly rated claimed; no score seen (Expedia/TripAdvisor/Google pages exist)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>+ family-friendly, gardens, kids area. - no cons seen</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rangadip%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>facebook; agoda h81757939</t>
         </is>
@@ -1078,12 +1174,25 @@
           <t>Phones conflict</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>No score (Facebook ~48k likes = followers, not rating)</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>+ view, kayaking, food, staff, kids' rides/pool. - none seen</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Nilanjana%20Boat%20Club%20and%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>avijatrik; offerong; tripbangla</t>
         </is>
@@ -1153,12 +1262,25 @@
           <t>No resort phone - use Facebook</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>No reviews on Take A Boat/Amarlodge</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>+ budget, lake view (YouTube titles). - unrated, no own phone</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Bargee%20Lake%20Valley%20Rangamati</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>amarlodge; takeaboat; adarbepari; trippainter; YouTube QktBTfqbYA8</t>
         </is>
@@ -1228,12 +1350,25 @@
           <t>Consistent</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor shared listing 4/5; one reviewer 9.5/10</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>+ secure Army-run, food 'best in Rangamati', lake view. - few activities, staff unhelpful, booking via Army contact, only ~11 rooms</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Aronnak%20Holiday%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>parjatanbd id 404; tripadvisor d7928494; bdbooking</t>
         </is>
@@ -1303,12 +1438,25 @@
           <t>Multiple numbers</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>No score seen</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>+ riverside, pods, kayaking, 20 AC rooms. - overpriced, rude waiters, cockroaches (snippets of reviews)</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Nisarga%20Pod%20House%20Kaptai</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t>dhakatribune; trip.com; hotels.com</t>
         </is>
@@ -1378,12 +1526,25 @@
           <t>Phone missing</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>16 of 19 reviews 5-star (platform not stated)</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>+ calm, food, camping, kayaking, bonfire. - 3 mixed reviews (details not found)</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Eco%20Valley</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>kaptaiecovalley.com; tourfo.com</t>
         </is>
@@ -1453,12 +1614,25 @@
           <t>FB snippet</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>+ riverside camping. - no reviews</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Kaptai%20Riverview%20Camping%20Point%20Kaptaimukh</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
@@ -1528,12 +1702,25 @@
           <t>Restricted</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>No numeric score</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>+ views, clean, seafood, helpful staff. - only 2 cottages; Navy/Army permission for overnight</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lake%20Paradise%20Kaptai</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>asiafirms d427221; lakeparadisebd.com</t>
         </is>
@@ -1603,12 +1790,25 @@
           <t>Reported open</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>- no reviews seen</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Green%20River%20View%20Kaptai%20Hotel</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr">
         <is>
           <t>facebook; vromonguide</t>
         </is>
@@ -1678,12 +1878,25 @@
           <t>Bangla snippet</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Google 4.0 (37 rev, via snippet)</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>- no details</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Happiness%20Hill%20Kaptai</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>agoda; vromontrips/goofly24 snippet</t>
         </is>
@@ -1753,12 +1966,25 @@
           <t>Exists</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Amarlodge: 0 reviews</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>- unrated</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rainya%20Tugun%20Eco%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>rainyatugun.com; tourtoday.com.bd</t>
         </is>
@@ -1828,12 +2054,25 @@
           <t>Contact via avijatrik</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>+ local-run cottages, tribal food (operator text). - no guest reviews</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Borgang%20Eco%20Cottage%20Rangamati</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>avijatrik.org/tour/borgang-eco-cottage-rangamati</t>
         </is>
@@ -1903,12 +2142,25 @@
           <t>Contact via FB</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Facebook: not yet rated (3 rev)</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>- unrated</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Rreng%20Lake%20Beach%20Resort%20Rangamati</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
@@ -1978,12 +2230,25 @@
           <t>Contact via FB</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor 3.7/5 (3 rev; restaurant)</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>+ local Hill Tracts food. Restaurant, not main lodging</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Gang%20Sabarang%20Rangamati</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
+      <c r="R20" s="2" t="inlineStr">
         <is>
           <t>tripadvisor d15141023</t>
         </is>
@@ -2053,12 +2318,25 @@
           <t>Exists</t>
         </is>
       </c>
-      <c r="N21" s="3" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Google 4.3 (3,247 rev); TripAdvisor 4.1 (17)</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>+ lakeside, pool, cafe, kids' rides. - power cuts, AC failure, dirty furniture, poor maintenance</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Polwel%20Park%20Rangamati</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>polwelpark.com; tripsilo</t>
         </is>
@@ -2128,12 +2406,25 @@
           <t>Consistent</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor 3/5 (19 rev; #1 of 2 inns)</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>+ lake-view balcony, clean new block, staff, cheap. - old block shabby, broken locks/AC</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Parjatan%20Holiday%20Complex%20Rangamati</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>hotels.gov.bd; parjatanbd id 816; wikimapia 17123711</t>
         </is>
@@ -2203,12 +2494,25 @@
           <t>Consistent</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Google 4.1 (321 rev, via snippet)</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>+ service, staff, clean, central. - none seen; hotel not lakeside</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Jum%20Palace%20Rangamati</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>jumpalace.com; parjatanbd id 401</t>
         </is>
@@ -2278,12 +2582,25 @@
           <t>Exists</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Top10Place 3.15/5</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>+ spacious, lake view, free breakfast+parking. - service 'okay'</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Shanghai%20International%20Rangamati</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>tour.com.bd; bdbooking; findglocal</t>
         </is>
@@ -2353,12 +2670,25 @@
           <t>Low confidence</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Not found (Facebook 4.2k likes)</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>- unrated</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Rajmahal%20International%20Rangamati</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="R25" s="2" t="inlineStr">
         <is>
           <t>facebook; amarlodge</t>
         </is>
@@ -2428,12 +2758,25 @@
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20City%20Rangamati</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2503,12 +2846,25 @@
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Hill%20Rangamati</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
+      <c r="R27" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2578,12 +2934,25 @@
           <t>Snippet only</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Forest%20Rest%20House%20Banarupa%20Rangamati</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
+      <c r="R28" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2653,12 +3022,25 @@
           <t>Listing only</t>
         </is>
       </c>
-      <c r="N29" s="3" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Facebook 100% recommend (7 rev)</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sonar%20Bangla%20Rangamati</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr">
+      <c r="R29" s="2" t="inlineStr">
         <is>
           <t>bangladeshhotels.net</t>
         </is>
@@ -2728,12 +3110,25 @@
           <t>Doubtful</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>TripAdvisor 2/5; Google 3.6 (441); PodSot 3.5 (453)</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>+ lakeside, cheap, restaurant. - quality concerns</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Green%20Castle%20Rangamati</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>bangladeshhotels.net</t>
         </is>
@@ -2803,12 +3198,25 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="N31" s="3" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>Names only</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Zoomking%20Eco%20Resort%20Kaptai</t>
         </is>
       </c>
-      <c r="O31" s="2" t="inlineStr">
+      <c r="R31" s="2" t="inlineStr">
         <is>
           <t>resortian (snippet); prothomalo b5frd0vwuj</t>
         </is>
@@ -2878,12 +3286,25 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="N32" s="3" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>Names only</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Hotel%20Sufia%20Rangamati</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="R32" s="2" t="inlineStr">
         <is>
           <t>vromonguide snippet</t>
         </is>
@@ -2892,67 +3313,67 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2964,7 +3385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2975,6 +3396,7 @@
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3018,6 +3440,11 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Guest feedback</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3060,6 +3487,11 @@
           <t>BEST houseboat fit for 30</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Press only; no guest reviews seen (8-room AC double-decker, on-board restaurant)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3102,6 +3534,11 @@
           <t>2D1N</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Facebook /reviews exists, no score; owner claims good feedback (unverified)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3144,6 +3581,11 @@
           <t>Small - would need multiple</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Facebook 1 review, no score</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3186,6 +3628,11 @@
           <t>Contact for 30-person quote</t>
         </is>
       </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3228,6 +3675,11 @@
           <t>Ask quote</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3270,6 +3722,11 @@
           <t>Lists Bargee, Royal Adventure</t>
         </is>
       </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3312,6 +3769,11 @@
           <t>Quote</t>
         </is>
       </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3354,6 +3816,11 @@
           <t>Quote</t>
         </is>
       </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3396,6 +3863,11 @@
           <t>Quote</t>
         </is>
       </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3438,6 +3910,11 @@
           <t>Quote</t>
         </is>
       </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3480,6 +3957,11 @@
           <t>Quote</t>
         </is>
       </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3522,6 +4004,11 @@
           <t>Need 2-3 boats for 30</t>
         </is>
       </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3562,6 +4049,11 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Get intercity quote</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -3576,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -3599,54 +4091,61 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>HARD LIMIT: Facebook, YouTube, Instagram, X, TripAdvisor, and nearly every travel blog/operator website were blocked from this environment. All data is from search-result snippets, not the pages themselves. YouTube/X yielded nothing.</t>
+          <t>Ratings sheet notes: ratings are from search-result snippets on the date shown, not opened pages; platforms differ in scale. Suitability score (1-5) is MY JUDGEMENT combining capacity for 30, price, transfer difficulty and review quality - not a platform rating.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Still 'Not found' after 3 rounds: WhatsApp numbers (except Rangatori), latitude/longitude, exact Google Maps place URLs, day-picnic/meal prices, most emails, Kaptai Eco Valley phone, Bargee's own phone, and operator phones for BD Cruise/GoZayaan/Galaxy/ITS/Avijatrik.</t>
+          <t>HARD LIMIT: Facebook, YouTube, Instagram, X, TripAdvisor, and nearly every travel blog/operator website were blocked from this environment. All data is from search-result snippets, not the pages themselves. YouTube/X yielded nothing.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Phones conflict for Lakeshore, Lake View Island, Divine Lake Island, Hill Taj, Nilanjana, Lake Paradise; 01911-060900 appears for both Nilanjana and Shukher Tori. Call and confirm before any advance payment.</t>
+          <t>Still 'Not found' after 3 rounds: WhatsApp numbers (except Rangatori), latitude/longitude, exact Google Maps place URLs, day-picnic/meal prices, most emails, Kaptai Eco Valley phone, Bargee's own phone, and operator phones for BD Cruise/GoZayaan/Galaxy/ITS/Avijatrik.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Google Maps links are name searches (no pin coordinates found) - verify the pin.</t>
+          <t>Phones conflict for Lakeshore, Lake View Island, Divine Lake Island, Hill Taj, Nilanjana, Lake Paradise; 01911-060900 appears for both Nilanjana and Shukher Tori. Call and confirm before any advance payment.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Prothom Alo reports ~20 resorts around the lake and only 3 with environmental clearance - ask about legal/permit status.</t>
+          <t>Google Maps links are name searches (no pin coordinates found) - verify the pin.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Some resorts are Army/Navy/Police-run; civilian overnight access may need permission.</t>
+          <t>Prothom Alo reports ~20 resorts around the lake and only 3 with environmental clearance - ask about legal/permit status.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Pages worth opening on your own network to fill the gaps: vromonguide.com/hotels-and-resorts-in-rangamati, bd-info.com/rangamati-hotel-resort-list, ratekom.com list, goofly24 Kaptai list, travelvibe.net/rangamati-hotels-list, resortian.com/blog/kaptai-lake-resorts, each resort's Facebook About page.</t>
+          <t>Some resorts are Army/Navy/Police-run; civilian overnight access may need permission.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Pages worth opening on your own network to fill the gaps: vromonguide.com/hotels-and-resorts-in-rangamati, bd-info.com/rangamati-hotel-resort-list, ratekom.com list, goofly24 Kaptai list, travelvibe.net/rangamati-hotels-list, resortian.com/blog/kaptai-lake-resorts, each resort's Facebook About page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Shortlist for 30: Lakeshore (whole resort) ; Royal Adventure houseboat (32 cap.) ; Kaptai Eco Valley (camping) ; Parjatan Holiday Complex ; or split groups across e.g. Aronnak + Divine Lake Island / Wildwood.</t>
         </is>

</xml_diff>